<commit_message>
Updated existing code and source data
Renamed data sheet to "Data" and updated the corresponding code along with removed unused code.
</commit_message>
<xml_diff>
--- a/Commodity_Data.xlsx
+++ b/Commodity_Data.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\OneDrive\Documents\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B536412-B305-4E5D-9DC9-7BAF87AA0145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97E5286-05A6-4BF0-B68D-B28203069C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1DBAD3D6-EA21-4CA8-ACD3-E65D1F41F517}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1DBAD3D6-EA21-4CA8-ACD3-E65D1F41F517}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="3" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Data" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>